<commit_message>
Fin de la documentación
Se ha terminado de documentar el documento a falta de añadir referencias a la bibliografía y futuras correciones
</commit_message>
<xml_diff>
--- a/Documentación/Pruebas comparativas.xlsx
+++ b/Documentación/Pruebas comparativas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unexes-my.sharepoint.com/personal/rmartinrw_alumnos_unex_es/Documents/TFG/Documentación/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="112" documentId="11_AD4D2F04E46CFB4ACB3E2095D596F110683EDF08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1A8D347-2141-4E29-A0B9-5F6867093EC4}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="11_AD4D2F04E46CFB4ACB3E2095D596F110683EDF08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0554D116-8972-45E0-A206-025F076B6622}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>Paquetería</t>
   </si>
@@ -72,10 +72,13 @@
     <t>Precisión de la E-nose</t>
   </si>
   <si>
-    <t>V(s)-Z</t>
+    <t>&gt;</t>
   </si>
   <si>
-    <t>V(s)-N</t>
+    <t>T(s)-Z</t>
+  </si>
+  <si>
+    <t>T(s)-N</t>
   </si>
 </sst>
 </file>
@@ -166,7 +169,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -175,6 +177,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1056,7 +1061,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES"/>
-              <a:t>Velocidad en segundos</a:t>
+              <a:t>Tiempo en segundos</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1105,7 +1110,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>V(s)-Z</c:v>
+                  <c:v>T(s)-Z</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1191,7 +1196,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>V(s)-N</c:v>
+                  <c:v>T(s)-N</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3213,6 +3218,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3476,7 +3485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K7"/>
+  <dimension ref="B2:O26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.33203125" customWidth="1"/>
@@ -3485,14 +3494,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>5</v>
@@ -3501,7 +3510,7 @@
         <v>6</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>7</v>
@@ -3509,7 +3518,7 @@
       <c r="J2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3517,28 +3526,28 @@
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="7">
         <v>1</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="7">
         <v>6</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="7">
         <v>10</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="7">
         <v>1</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="7">
         <v>155</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="7">
         <v>3</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3546,28 +3555,28 @@
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="7">
         <v>1</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="7">
         <v>25</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="7">
         <v>10</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="7">
         <v>0</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="7">
         <v>440</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="7">
         <v>0</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3575,28 +3584,28 @@
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="7">
         <v>1</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="7">
         <v>15</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="7">
         <v>10</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="7">
         <v>0</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="7">
         <v>390</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="7">
         <v>3</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3604,28 +3613,28 @@
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="7">
         <v>1</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="7">
         <v>22</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="7">
         <v>10</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="7">
         <v>1</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="7">
         <v>170</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="7">
         <v>10</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3633,8 +3642,13 @@
       <c r="J7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="6" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="15:15" x14ac:dyDescent="0.3">
+      <c r="O26" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>